<commit_message>
Mitigate lumbar strain in June plan
</commit_message>
<xml_diff>
--- a/data/checkins/2026-06.template.xlsx
+++ b/data/checkins/2026-06.template.xlsx
@@ -113,9 +113,9 @@
 Adjusted: Shortened for schedule constraints. Light active commute counted. Adjusted for temporary low-back recovery constraint.
 Warm-up: 5-7 min easy bike, band pull-aparts, scap push-ups, and 2 bench ramp sets.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
-Bench press: top set 1 x 4-6 at RPE 8, then 3 back-off sets x 5-7 at RPE 7-8.
-Pull-ups: 4 x 4-8 at RPE 8 paired with chest-supported row 4 x 8-12 at RPE 8.
-Incline dumbbell press: 3 x 8-12 at RPE 8 paired with dips or push-ups 2-3 x clean reps, stop at 1-2 RIR.
+Bench press: top set 1 x 4-6 at RPE 6-7, then 3 back-off sets x 5-7 at RPE 6-7.
+Pull-ups: 4 x 4-8 at RPE 6-7 paired with chest-supported row 4 x 8-12 at RPE 6-7.
+Incline dumbbell press: 3 x 8-12 at RPE 6-7 paired with dips or push-ups 2-3 x clean reps, stop at 1-2 RIR.
 Core finisher: Pallof press 3 x 10 per side plus dead bug 2 x 8 per side; keep the trunk quiet and pain-free. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
         </is>
       </c>
@@ -130,7 +130,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="241" customHeight="1">
+    <row r="3" ht="256" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>2026-06-02 - Lower Strength + Knee Capacity</t>
@@ -142,9 +142,9 @@
 Adjusted: Shortened for schedule constraints. Light active commute counted. Adjusted for temporary low-back recovery constraint.
 Warm-up: 7-8 min bike, ankle rocks, bodyweight squats, and tibialis raises.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
-Hack squat or goblet squat: top set 1 x 6-8 at RPE 8, then 3 back-off sets x 8-10 at RPE 7-8.
+Hack squat, leg press, or supported split squat: 3 x 6-10 at RPE 6-7; stop if symptoms rise.
 Back-friendly posterior chain: seated or lying leg curl 3 x 10-15 at RPE 6-7, plus bodyweight glute bridge 2 x 12 if symptom-free.
-Split squat or step-up: 3 x 8-10 per leg at RPE 7 paired with leg curl 3 x 10-15 at RPE 8.
+Supported split squat or step-up: 2-3 x 8-10 per leg at RPE 6-7 paired with leg curl 2-3 x 10-15 at RPE 6-7.
 Core finisher: calf raises plus tibialis raises 4 x 12-20 each at RPE 7, then side plank 2 x 30 sec. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
         </is>
       </c>
@@ -197,11 +197,11 @@
           <t xml:space="preserve">Macros: 3350 kcal, 165 g protein, 455 g carbs, 95 g fat
 Adjusted: Adjusted for moderate recovery constraint. Light active commute counted. Adjusted for temporary low-back recovery constraint.
 Warm-up: 5 min easy cardio, shoulder circles, light rows, and scap pull-ups.
-Progression: double progression; beat total quality reps before adding load or a set, keeping most work at RPE 8-9. Moderate recovery constraint: reduce volume by 25-40%, cap hard sets at RPE 7, and leave the gym/run fresher than planned. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
-Pull-ups: 5 x 4-8 or 20-30 total quality reps at RPE 8.
-Dips or push-ups: 3 x 8-15 at RPE 8-9, stop before shoulder position changes.
-One-arm dumbbell row or inverted row: 3 x 8-12 at RPE 8 paired with incline dumbbell press 2-3 x 8-12 at RPE 8.
-Core finisher: lateral raises plus hanging leg raises 2-3 sets each at RPE 8. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
+Progression: double progression; beat total quality reps before adding load or a set, keeping most work at RPE 6-7. Moderate recovery constraint: reduce volume by 25-40%, cap hard sets at RPE 7, and leave the gym/run fresher than planned. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
+Pull-ups: 5 x 4-8 or 20-30 total quality reps at RPE 6-7.
+Dips or push-ups: 3 x 8-15 at RPE 6-7, stop before shoulder position changes.
+One-arm dumbbell row or inverted row: 3 x 8-12 at RPE 6-7 paired with incline dumbbell press 2-3 x 8-12 at RPE 6-7.
+Core finisher: lateral raises plus hanging leg raises 2-3 sets each at RPE 6-7. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -254,9 +254,9 @@
           <t xml:space="preserve">Macros: 3550 kcal, 165 g protein, 520 g carbs, 100 g fat
 Adjusted: Adjusted for temporary low-back recovery constraint.
 Warm-up jog: 10-12 min easy plus leg swings, A-skips, ankling, and 3 relaxed strides.
-Progression: add sprint reps only when contacts stay snappy and knees stay quiet the next day; sprint RPE 7-8, never max. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
+Progression: add sprint reps only when contacts stay snappy and knees stay quiet the next day; sprint RPE 6-7, never max. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
 Plyometrics: pogos 3 x 20 sec, snap-downs 3 x 5, snap-downs 2 x 5 at crisp RPE 6-7.
-Hill sprints: 6 x 10-12 sec uphill at sprint RPE 7-8; full walk-back recovery.
+Hill sprints: 6 x 10-12 sec uphill at sprint RPE 6-7; full walk-back recovery.
 Stop the sprint set if mechanics get sloppy or knees feel sharp.
 Optional: dead bug 3 x 8 per side and side plank 2 x 30 sec. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
         </is>
@@ -312,9 +312,9 @@
 Warm-up: 7 min easy cardio, squat-to-stand, band rows, push-ups, and hinge ramp sets.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
 Incline press or bench press: top set 1 x 6-8 at RPE 8, then 3-4 back-off sets x 8-10 at RPE 7-8.
-Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; no deadlifts or hyperextensions; start lightly.
+Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; skip loaded hinges and back-extension work; start lightly.
 Pull-ups or chest-supported rows: 4 x 6-10 at RPE 8 paired with goblet squat 3 x 8-12 at RPE 7.
-Core finisher: farmer carries 3 x 40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: farmer carries 3 x 40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -355,7 +355,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="226" customHeight="1">
+    <row r="11" ht="241" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>2026-06-10 - Lower Unilateral + Posterior Chain</t>
@@ -368,9 +368,9 @@
 Warm-up: 7-8 min bike, split squat isometric holds, ankle rocks, and hinge ramp sets.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
 Bulgarian split squat or step-up: 3-4 x 6-10 per leg at RPE 7-8.
-Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; no deadlifts or hyperextensions; start lightly.
+Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; skip loaded hinges and back-extension work; start lightly.
 Walking lunges: 2-3 x 12 steps per leg at RPE 7.
-Core finisher: calf raises plus Copenhagen plank 2-3 sets each at RPE 7. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: calf raises plus Copenhagen plank 2-3 sets each at RPE 7. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -384,7 +384,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="196" customHeight="1">
+    <row r="12" ht="211" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>2026-06-11 - Calisthenics Density + Zone 2 (4 km run)</t>
@@ -399,7 +399,7 @@
 Density block: 20 min alternating pull-ups, push-ups, inverted rows, and hanging knee raises at 2 RIR.
 Easy run RPE 3-4: 4 km conversational immediately after or in the morning.
 Carry finisher: suitcase carry 3 x 30 m per side at RPE 7.
-Optional: lateral raises or curls 2 x 15-20 at RPE 8 if time remains. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Optional: lateral raises or curls 2 x 15-20 at RPE 8 if time remains. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -456,7 +456,7 @@
 Plyometrics: pogos 3 x 20 sec, low broad jumps 4 x 2, and med-ball slams 4 x 5 at crisp RPE 6-7 if available.
 Hill sprint technique: 4-6 x 8-10 sec at sprint RPE 7-8.
 Functional work: sled push if easy to set up or farmer carries 4 x 30 m at RPE 7. Keep carries light and skip them if the low back feels loaded.
-Core: crawling 3 x 20 m or dead bug 3 x 8 per side. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core: crawling 3 x 20 m or dead bug 3 x 8 per side. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -512,7 +512,7 @@
 Bench press: top set 1 x 4-6 at RPE 8, then 3 back-off sets x 5-7 at RPE 7-8.
 Pull-ups: 4 x 4-8 at RPE 8 paired with chest-supported row 4 x 8-12 at RPE 8.
 Incline dumbbell press: 3 x 8-12 at RPE 8 paired with dips or push-ups 2-3 x clean reps, stop at 1-2 RIR.
-Core finisher: farmer carries 4 x 30-40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: farmer carries 4 x 30-40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -539,9 +539,9 @@
 Warm-up: 7-8 min bike, ankle rocks, bodyweight squats, and tibialis raises.
 Progression: double progression; add load only when knee tracking stays clean, discomfort stays 0-2/10, and top sets stay near RPE 8. Reduce volume by 25-40% before adding intensity. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
 Hack squat or goblet squat: top set 1 x 6-8 at RPE 8, then 3 back-off sets x 8-10 at RPE 7-8.
-Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; no deadlifts or hyperextensions; start lightly.
+Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; skip loaded hinges and back-extension work; start lightly.
 Split squat or step-up: 3 x 8-10 per leg at RPE 7 paired with leg curl 3 x 10-15 at RPE 8.
-Core finisher: calf raises plus tibialis raises 4 x 12-20 each at RPE 7, then side plank 2 x 30 sec. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: calf raises plus tibialis raises 4 x 12-20 each at RPE 7, then side plank 2 x 30 sec. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -597,7 +597,7 @@
 Pull-ups: 5 x 4-8 or 20-30 total quality reps at RPE 8.
 Dips or push-ups: 3 x 8-15 at RPE 8-9, stop before shoulder position changes.
 One-arm dumbbell row or inverted row: 3 x 8-12 at RPE 8 paired with incline dumbbell press 2-3 x 8-12 at RPE 8.
-Core finisher: lateral raises plus hanging leg raises 2-3 sets each at RPE 8. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: lateral raises plus hanging leg raises 2-3 sets each at RPE 8. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -654,7 +654,7 @@
 Plyometrics: pogos 3 x 20 sec, snap-downs 3 x 5, low broad jumps 3 x 3 at crisp RPE 6-7.
 Hill sprints: 6 x 10-12 sec uphill at sprint RPE 7-8; full walk-back recovery.
 Stop the sprint set if mechanics get sloppy or knees feel sharp.
-Optional: dead bug 3 x 8 per side and side plank 2 x 30 sec. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Optional: dead bug 3 x 8 per side and side plank 2 x 30 sec. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -708,9 +708,9 @@
 Warm-up: 7 min easy cardio, squat-to-stand, band rows, push-ups, and hinge ramp sets.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
 Incline press or bench press: top set 1 x 6-8 at RPE 8, then 3-4 back-off sets x 8-10 at RPE 7-8.
-Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; no deadlifts or hyperextensions; start lightly.
+Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; skip loaded hinges and back-extension work; start lightly.
 Pull-ups or chest-supported rows: 4 x 6-10 at RPE 8 paired with goblet squat 3 x 8-12 at RPE 7.
-Core finisher: farmer carries 3 x 40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: farmer carries 3 x 40 m at RPE 7 plus dead bug 2 x 8 per side. Keep carries light and skip them if the low back feels loaded. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -751,7 +751,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="226" customHeight="1">
+    <row r="25" ht="241" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>2026-06-24 - Lower Unilateral + Posterior Chain</t>
@@ -764,9 +764,9 @@
 Warm-up: 7-8 min bike, split squat isometric holds, ankle rocks, and hinge ramp sets.
 Progression: use the minimum effective dose today; complete the first 3 main lifts and add accessories only if energy is good. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
 Bulgarian split squat or step-up: 3-4 x 6-10 per leg at RPE 7-8.
-Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; no deadlifts or hyperextensions; start lightly.
+Back-friendly posterior chain: hip thrust, glute bridge, or leg curl 3 x 8-12 at RPE 6-7; skip loaded hinges and back-extension work; start lightly.
 Walking lunges: 2-3 x 12 steps per leg at RPE 7.
-Core finisher: calf raises plus Copenhagen plank 2-3 sets each at RPE 7. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Core finisher: calf raises plus Copenhagen plank 2-3 sets each at RPE 7. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -780,7 +780,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="226" customHeight="1">
+    <row r="26" ht="241" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>2026-06-25 - Calisthenics Density + Zone 2 (4 km run)</t>
@@ -795,7 +795,7 @@
 Density block: 20 min alternating pull-ups, push-ups, inverted rows, and hanging knee raises at 2 RIR.
 Easy run RPE 3-4: 4 km conversational immediately after or in the morning.
 Carry finisher: suitcase carry 3 x 30 m per side at RPE 7.
-Optional: lateral raises or curls 2 x 15-20 at RPE 8 if time remains. Low-back ramp: no deadlifts or hyperextensions; start lightly and keep supported posterior-chain work pain-free.</t>
+Optional: lateral raises or curls 2 x 15-20 at RPE 8 if time remains. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">

</xml_diff>

<commit_message>
Prioritize gym frequency in hybrid wave
</commit_message>
<xml_diff>
--- a/data/checkins/2026-06.template.xlsx
+++ b/data/checkins/2026-06.template.xlsx
@@ -215,21 +215,22 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="136" customHeight="1">
+    <row r="6" ht="226" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-05 - Recovery + Knee Capacity</t>
+          <t>2026-06-05 - Accessory Strength + Knee/Core Capacity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
+          <t xml:space="preserve">Macros: 3350 kcal, 165 g protein, 455 g carbs, 95 g fat
 Adjusted: Adjusted for temporary low-back recovery constraint.
-Recovery RPE 2-3: 30-45 min walk or easy bike; keep legs fresh for the next sprint exposure.
-Knee capacity: tibialis raises 2 x 20, slow calf raises 2 x 15, and wall sit 2 x 30-45 sec at RPE 6-7.
-Mobility: hips, ankles, quads, calves, and glutes for 10-12 min.
-Core: Pallof press or side plank 2-3 easy sets.
-Fueling: keep protein fixed and include carbs at lunch and dinner.</t>
+Warm-up: 5-7 min easy bike, shoulder prep, ankle rocks, and light calf raises.
+Progression: gym priority exposure without recovery debt; keep all work at RPE 6-7, leave 3 RIR, and finish fresher than a normal strength day. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
+Chest-supported row or cable row: 3 x 10-12 at RPE 7 paired with machine shoulder press or lateral raises 3 x 10-15 at RPE 7.
+Knee capacity: seated or lying leg curl 2-3 x 12-15, tibialis raises 2 x 20, slow calf raises 2 x 15, and wall sit 2 x 30-45 sec at RPE 6-7.
+Arms and upper pump: curls plus triceps pressdowns or push-ups 2 x 10-15 at RPE 6-7.
+Core: Pallof press or side plank 2-3 easy sets, then 8-10 min hips, ankles, quads, and calves. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -255,7 +256,7 @@
 Adjusted: Adjusted for temporary low-back recovery constraint.
 Warm-up jog: 10-12 min easy plus leg swings, A-skips, ankling, and 3 relaxed strides.
 Progression: add sprint reps only when contacts stay snappy and knees stay quiet the next day; sprint RPE 6-7, never max. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
-Plyometrics: pogos 3 x 20 sec, snap-downs 3 x 5, snap-downs 2 x 5 at crisp RPE 6-7.
+Plyometrics: pogos 3 x 20 sec and snap-downs 3 x 5 at crisp RPE 6-7.
 Hill sprints: 6 x 10-12 sec uphill at sprint RPE 6-7; full walk-back recovery.
 Stop the sprint set if mechanics get sloppy or knees feel sharp.
 Optional: dead bug 3 x 8 per side and side plank 2 x 30 sec. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
@@ -611,21 +612,22 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="136" customHeight="1">
+    <row r="20" ht="226" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-19 - Recovery + Knee Capacity</t>
+          <t>2026-06-19 - Accessory Strength + Knee/Core Capacity</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
-Adjusted: Back-friendly loading ramp.
-Recovery RPE 2-3: 30-45 min walk or easy bike; keep legs fresh for the next sprint exposure.
-Knee capacity: tibialis raises 2 x 20, slow calf raises 2 x 15, and wall sit 2 x 30-45 sec at RPE 6-7.
-Mobility: hips, ankles, quads, calves, and glutes for 10-12 min.
-Core: Pallof press or side plank 2-3 easy sets.
-Fueling: keep protein fixed and include carbs at lunch and dinner.</t>
+          <t xml:space="preserve">Macros: 3350 kcal, 165 g protein, 455 g carbs, 95 g fat
+Adjusted: Adjusted for schedule constraints. Back-friendly loading ramp.
+Warm-up: 5-7 min easy bike, shoulder prep, ankle rocks, and light calf raises.
+Progression: gym priority exposure without recovery debt; keep all work at RPE 6-7, leave 3 RIR, and finish fresher than a normal strength day. Reduce volume by 25-40% before adding intensity. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
+Chest-supported row or cable row: 3 x 10-12 at RPE 7 paired with machine shoulder press or lateral raises 3 x 10-15 at RPE 7.
+Knee capacity: seated or lying leg curl 2-3 x 12-15, tibialis raises 2 x 20, slow calf raises 2 x 15, and wall sit 2 x 30-45 sec at RPE 6-7.
+Arms and upper pump: curls plus triceps pressdowns or push-ups 2 x 10-15 at RPE 7-8.
+Core: Pallof press or side plank 2-3 easy sets, then 8-10 min hips, ankles, quads, and calves. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">

</xml_diff>

<commit_message>
Apply June schedule overrides
</commit_message>
<xml_diff>
--- a/data/checkins/2026-06.template.xlsx
+++ b/data/checkins/2026-06.template.xlsx
@@ -186,22 +186,21 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="256" customHeight="1">
+    <row r="5" ht="136" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-04 - Upper Calisthenics + Hypertrophy</t>
+          <t>2026-06-04 - Unavailable / No Workout</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3350 kcal, 165 g protein, 455 g carbs, 95 g fat
-Adjusted: Adjusted for moderate recovery constraint. Light active commute counted. Adjusted for temporary low-back recovery constraint.
-Warm-up: 5 min easy cardio, shoulder circles, light rows, and scap pull-ups.
-Progression: double progression; beat total quality reps before adding load or a set, keeping most work at RPE 6-7. Moderate recovery constraint: reduce volume by 25-40%, cap hard sets at RPE 7, and leave the gym/run fresher than planned. Light active commute: 30 min calm cycling each way counts as easy aerobic load; keep hard sets at the prescribed RPE. Temporary low-back recovery constraint: cap loaded work at RPE 6-7 and stop if symptoms rise.
-Pull-ups: 5 x 4-8 or 20-30 total quality reps at RPE 6-7.
-Dips or push-ups: 3 x 8-15 at RPE 6-7, stop before shoulder position changes.
-One-arm dumbbell row or inverted row: 3 x 8-12 at RPE 6-7 paired with incline dumbbell press 2-3 x 8-12 at RPE 6-7.
-Core finisher: lateral raises plus hanging leg raises 2-3 sets each at RPE 6-7. Temporary low-back recovery constraint: avoid loaded hinging and heavy bracing; use machines or supported positions where possible.</t>
+          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
+Adjusted: No scheduled workout.
+Warm-up: none; this is a no-workout day.
+No scheduled workout today because the day is unavailable.
+Keep the plan simple: normal walking only, basic mobility if convenient, and enough food to avoid under-fueling.
+Fueling: normal meals, protein target, and no intentional calorie restriction.
+Recovery priority: sleep, hydration, and an easy protein target.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -641,22 +640,22 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="196" customHeight="1">
+    <row r="21" ht="166" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-20 - Plyometrics + Hill Sprint Technique (3 km run)</t>
+          <t>2026-06-20 - Early Easier Morning Strength</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3550 kcal, 165 g protein, 520 g carbs, 100 g fat
-Adjusted: Adjusted for moderate recovery constraint. Back-friendly loading ramp.
-Warm-up jog: 10-12 min easy plus leg swings, A-skips, ankling, and 3 relaxed strides.
-Progression: add sprint reps only when contacts stay snappy and knees stay quiet the next day; sprint RPE 7-8, never max. Moderate recovery constraint: reduce volume by 25-40%, cap hard sets at RPE 7, and leave the gym/run fresher than planned. Low-back ramp: start lightly and add load only when the next morning is symptom-free.
-Plyometrics: pogos 3 x 20 sec, snap-downs 3 x 5, low broad jumps 3 x 3 at crisp RPE 6-7.
-Hill sprints: 6 x 10-12 sec uphill at sprint RPE 7-8; full walk-back recovery.
-Stop the sprint set if mechanics get sloppy or knees feel sharp.
-Optional: dead bug 3 x 8 per side and side plank 2 x 30 sec. Low-back ramp: skip loaded hinges and back-extension work; start lightly and keep supported posterior-chain work pain-free.</t>
+          <t xml:space="preserve">Macros: 3350 kcal, 165 g protein, 455 g carbs, 95 g fat
+Adjusted: Moved to an early easier morning workout.
+Timing: early morning session before the day gets busy.
+Warm-up: 5 min easy bike plus shoulder, hip, and ankle prep.
+Main work: bench press 3 x 5 at RPE 6-7, chest-supported row 3 x 8-10 at RPE 7, and leg press or goblet squat 2 x 8 at RPE 6.
+Accessories: lateral raises 2 x 15, curls 2 x 12, and Pallof press 2 x 10 per side.
+Fueling: eat a small carb-focused breakfast or snack before training, then a normal protein-rich meal after.
+Stop while fresh; this is an easier session, not a progression test.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -840,20 +839,22 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="121" customHeight="1">
+    <row r="28" ht="151" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06-27 - Recovery / Maintenance Day (3 km run)</t>
+          <t>2026-06-27 - Festival Walking + No Workout</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
-Adjusted: Adjusted for high-risk schedule constraints. Back-friendly loading ramp.
-Keep training conservative because the private calendar review found a high-risk schedule constraint.
-Main work: 30-60 min walk or easy bike, then 10-12 min mobility.
-Optional: light pump circuit only if sleep, hydration, and joints feel normal.
-Recovery: protein target stays fixed; prioritize fluids, sodium, and carbohydrate-dense meals.</t>
+          <t xml:space="preserve">Macros: 3400 kcal, 165 g protein, 500 g carbs, 80 g fat
+Adjusted: No scheduled workout; high walking load counted.
+Warm-up: none; festival walking is the day's physical load.
+No gym, running, sprinting, plyometrics, or calisthenics session today.
+Expected load: 20,000+ steps from festival walking; count that as the training stress.
+Fueling: prioritize fluids, sodium, protein when practical, and carbohydrate-dense meals.
+Recovery priority: hydrate early, add sodium, get protein when practical, and use carbohydrate-dense meals.
+Do not try to make up missed sessions during the festival block.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -867,19 +868,22 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="91" customHeight="1">
+    <row r="29" ht="151" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-28 - Recovery Day After High-Risk Schedule (3 km run)</t>
+          <t>2026-06-28 - Festival Walking + No Workout</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
-Adjusted: Adjusted after high-risk schedule constraints. Back-friendly loading ramp.
-No heavy lower body or hard running today.
-Recovery: 30-60 min walk, 10 min mobility, hydration, sodium, and easy meals with carbs.
-Optional: light upper accessories only if energy is clearly good.</t>
+          <t xml:space="preserve">Macros: 3400 kcal, 165 g protein, 500 g carbs, 80 g fat
+Adjusted: No scheduled workout; high walking load counted.
+Warm-up: none; festival walking is the day's physical load.
+No gym, running, sprinting, plyometrics, or calisthenics session today.
+Expected load: 20,000+ steps from festival walking; count that as the training stress.
+Fueling: prioritize fluids, sodium, protein when practical, and carbohydrate-dense meals.
+Recovery priority: hydrate early, add sodium, get protein when practical, and use carbohydrate-dense meals.
+Do not try to make up missed sessions during the festival block.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -893,20 +897,22 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="121" customHeight="1">
+    <row r="30" ht="151" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-29 - Recovery / Maintenance Day</t>
+          <t>2026-06-29 - Festival Walking + No Workout</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3200 kcal, 165 g protein, 400 g carbs, 105 g fat
-Adjusted: Adjusted for high-risk schedule constraints. Back-friendly loading ramp.
-Keep training conservative because the private calendar review found a high-risk schedule constraint.
-Main work: 30-60 min walk or easy bike, then 10-12 min mobility.
-Optional: light pump circuit only if sleep, hydration, and joints feel normal.
-Recovery: protein target stays fixed; prioritize fluids, sodium, and carbohydrate-dense meals.</t>
+          <t xml:space="preserve">Macros: 3400 kcal, 165 g protein, 500 g carbs, 80 g fat
+Adjusted: No scheduled workout; high walking load counted.
+Warm-up: none; festival walking is the day's physical load.
+No gym, running, sprinting, plyometrics, or calisthenics session today.
+Expected load: 20,000+ steps from festival walking; count that as the training stress.
+Fueling: prioritize fluids, sodium, protein when practical, and carbohydrate-dense meals.
+Recovery priority: hydrate early, add sodium, get protein when practical, and use carbohydrate-dense meals.
+Do not try to make up missed sessions during the festival block.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -920,19 +926,22 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="91" customHeight="1">
+    <row r="31" ht="151" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-30 - Recovery Day After High-Risk Schedule</t>
+          <t>2026-06-30 - Festival Walking + No Workout</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Macros: 3150 kcal, 165 g protein, 385 g carbs, 105 g fat
-Adjusted: Adjusted after high-risk schedule constraints. Back-friendly loading ramp.
-No heavy lower body or hard running today.
-Recovery: 30-60 min walk, 10 min mobility, hydration, sodium, and easy meals with carbs.
-Optional: light upper accessories only if energy is clearly good.</t>
+          <t xml:space="preserve">Macros: 3400 kcal, 165 g protein, 500 g carbs, 80 g fat
+Adjusted: No scheduled workout; high walking load counted.
+Warm-up: none; festival walking is the day's physical load.
+No gym, running, sprinting, plyometrics, or calisthenics session today.
+Expected load: 20,000+ steps from festival walking; count that as the training stress.
+Fueling: prioritize fluids, sodium, protein when practical, and carbohydrate-dense meals.
+Recovery priority: hydrate early, add sodium, get protein when practical, and use carbohydrate-dense meals.
+Do not try to make up missed sessions during the festival block.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">

</xml_diff>